<commit_message>
update exporting to excel to properly use styles
</commit_message>
<xml_diff>
--- a/natural-language-processing/exports/mia07_t3_tra_resultados_viterbi.xlsx
+++ b/natural-language-processing/exports/mia07_t3_tra_resultados_viterbi.xlsx
@@ -26,12 +26,17 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007FFFD4"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +51,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -473,7 +479,7 @@
       <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="1" t="n">
         <v>1.295582484193506e-09</v>
       </c>
       <c r="F2" t="n">
@@ -495,7 +501,7 @@
           <t>VMIP3S0</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="1" t="n">
         <v>0.0012941074971961</v>
       </c>
       <c r="C3" t="n">
@@ -529,7 +535,7 @@
       <c r="B4" t="n">
         <v>0</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="1" t="n">
         <v>1.988063133517315e-05</v>
       </c>
       <c r="D4" t="n">
@@ -541,7 +547,7 @@
       <c r="F4" t="n">
         <v>0</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="1" t="n">
         <v>5.440257583147429e-12</v>
       </c>
       <c r="H4" t="n">
@@ -575,7 +581,7 @@
       <c r="G5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="1" t="n">
         <v>4.107075865754602e-15</v>
       </c>
       <c r="I5" t="n">
@@ -631,7 +637,7 @@
       <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="1" t="n">
         <v>6.385259012197449e-11</v>
       </c>
       <c r="G7" t="n">
@@ -671,7 +677,7 @@
       <c r="H8" t="n">
         <v>0</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="1" t="n">
         <v>3.529518322132861e-16</v>
       </c>
     </row>
@@ -690,7 +696,7 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="1" t="n">
         <v>2.827818374535177e-08</v>
       </c>
       <c r="F9" t="n">
@@ -718,7 +724,7 @@
       <c r="C10" t="n">
         <v>0</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="1" t="n">
         <v>2.779888150251198e-06</v>
       </c>
       <c r="E10" t="n">

</xml_diff>